<commit_message>
refactor: simplify GRW template + fix output path + add markup %
</commit_message>
<xml_diff>
--- a/modules/po_tools/grw_invoice_converter/output/Cafe Monarch GRW S58672.xlsx
+++ b/modules/po_tools/grw_invoice_converter/output/Cafe Monarch GRW S58672.xlsx
@@ -878,24 +878,24 @@
         <v>1</v>
       </c>
       <c r="I2" s="9" t="n">
-        <v>695</v>
+        <v>1</v>
       </c>
       <c r="J2" s="60" t="n">
         <v>695</v>
       </c>
       <c r="K2" s="61" t="n">
-        <v>1</v>
+        <v>800</v>
       </c>
       <c r="L2" s="9" t="n">
         <v>800</v>
       </c>
-      <c r="M2" s="62" t="n">
+      <c r="M2" s="62" t="n"/>
+      <c r="N2" s="60" t="n">
         <v>695</v>
       </c>
-      <c r="N2" s="60" t="n">
-        <v>800</v>
-      </c>
-      <c r="O2" s="60" t="n"/>
+      <c r="O2" s="60" t="n">
+        <v>695</v>
+      </c>
       <c r="P2" s="13" t="n"/>
       <c r="Q2" s="61" t="n"/>
       <c r="R2" s="63" t="n"/>
@@ -924,24 +924,24 @@
         <v>1</v>
       </c>
       <c r="I3" s="9" t="n">
-        <v>550</v>
+        <v>1</v>
       </c>
       <c r="J3" s="60" t="n">
         <v>550</v>
       </c>
       <c r="K3" s="61" t="n">
-        <v>1</v>
+        <v>633</v>
       </c>
       <c r="L3" s="9" t="n">
         <v>633</v>
       </c>
-      <c r="M3" s="62" t="n">
+      <c r="M3" s="62" t="n"/>
+      <c r="N3" s="60" t="n">
         <v>550</v>
       </c>
-      <c r="N3" s="60" t="n">
-        <v>633</v>
-      </c>
-      <c r="O3" s="60" t="n"/>
+      <c r="O3" s="60" t="n">
+        <v>550</v>
+      </c>
       <c r="P3" s="13" t="n"/>
       <c r="Q3" s="61" t="n"/>
       <c r="R3" s="63" t="n"/>
@@ -970,24 +970,24 @@
         <v>1</v>
       </c>
       <c r="I4" s="9" t="n">
-        <v>1395</v>
+        <v>1</v>
       </c>
       <c r="J4" s="60" t="n">
         <v>1395</v>
       </c>
       <c r="K4" s="61" t="n">
-        <v>1</v>
+        <v>1605</v>
       </c>
       <c r="L4" s="9" t="n">
         <v>1605</v>
       </c>
-      <c r="M4" s="62" t="n">
+      <c r="M4" s="62" t="n"/>
+      <c r="N4" s="60" t="n">
         <v>1395</v>
       </c>
-      <c r="N4" s="60" t="n">
-        <v>1605</v>
-      </c>
-      <c r="O4" s="60" t="n"/>
+      <c r="O4" s="60" t="n">
+        <v>1395</v>
+      </c>
       <c r="P4" s="13" t="n"/>
       <c r="Q4" s="61" t="n"/>
       <c r="R4" s="63" t="n"/>
@@ -1016,24 +1016,24 @@
         <v>1</v>
       </c>
       <c r="I5" s="9" t="n">
-        <v>285</v>
+        <v>1</v>
       </c>
       <c r="J5" s="60" t="n">
         <v>285</v>
       </c>
       <c r="K5" s="61" t="n">
-        <v>1</v>
+        <v>328</v>
       </c>
       <c r="L5" s="9" t="n">
         <v>328</v>
       </c>
-      <c r="M5" s="62" t="n">
+      <c r="M5" s="62" t="n"/>
+      <c r="N5" s="60" t="n">
         <v>285</v>
       </c>
-      <c r="N5" s="60" t="n">
-        <v>328</v>
-      </c>
-      <c r="O5" s="60" t="n"/>
+      <c r="O5" s="60" t="n">
+        <v>285</v>
+      </c>
       <c r="P5" s="13" t="n"/>
       <c r="Q5" s="61" t="n"/>
       <c r="R5" s="63" t="n"/>
@@ -1062,24 +1062,24 @@
         <v>1</v>
       </c>
       <c r="I6" s="9" t="n">
-        <v>1044.75</v>
+        <v>1</v>
       </c>
       <c r="J6" s="60" t="n">
         <v>1044.75</v>
       </c>
       <c r="K6" s="61" t="n">
-        <v>1</v>
+        <v>1145</v>
       </c>
       <c r="L6" s="9" t="n">
         <v>1145</v>
       </c>
-      <c r="M6" s="62" t="n">
+      <c r="M6" s="62" t="n"/>
+      <c r="N6" s="60" t="n">
         <v>1044.75</v>
       </c>
-      <c r="N6" s="60" t="n">
-        <v>1145</v>
-      </c>
-      <c r="O6" s="60" t="n"/>
+      <c r="O6" s="60" t="n">
+        <v>1044.75</v>
+      </c>
       <c r="P6" s="13" t="n"/>
       <c r="Q6" s="61" t="n"/>
       <c r="R6" s="63" t="n"/>
@@ -1108,24 +1108,24 @@
         <v>1</v>
       </c>
       <c r="I7" s="9" t="n">
-        <v>1254.75</v>
+        <v>1</v>
       </c>
       <c r="J7" s="60" t="n">
         <v>1254.75</v>
       </c>
       <c r="K7" s="61" t="n">
-        <v>1</v>
+        <v>1375</v>
       </c>
       <c r="L7" s="9" t="n">
         <v>1375</v>
       </c>
-      <c r="M7" s="62" t="n">
+      <c r="M7" s="62" t="n"/>
+      <c r="N7" s="60" t="n">
         <v>1254.75</v>
       </c>
-      <c r="N7" s="60" t="n">
-        <v>1375</v>
-      </c>
-      <c r="O7" s="60" t="n"/>
+      <c r="O7" s="60" t="n">
+        <v>1254.75</v>
+      </c>
       <c r="P7" s="13" t="n"/>
       <c r="Q7" s="61" t="n"/>
       <c r="R7" s="63" t="n"/>
@@ -1154,24 +1154,24 @@
         <v>1</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>1312.5</v>
+        <v>1</v>
       </c>
       <c r="J8" s="60" t="n">
         <v>1312.5</v>
       </c>
       <c r="K8" s="61" t="n">
-        <v>1</v>
+        <v>1438</v>
       </c>
       <c r="L8" s="9" t="n">
         <v>1438</v>
       </c>
-      <c r="M8" s="62" t="n">
+      <c r="M8" s="62" t="n"/>
+      <c r="N8" s="60" t="n">
         <v>1312.5</v>
       </c>
-      <c r="N8" s="60" t="n">
-        <v>1438</v>
-      </c>
-      <c r="O8" s="60" t="n"/>
+      <c r="O8" s="60" t="n">
+        <v>1312.5</v>
+      </c>
       <c r="P8" s="13" t="n"/>
       <c r="Q8" s="61" t="n"/>
       <c r="R8" s="63" t="n"/>
@@ -1200,24 +1200,24 @@
         <v>3</v>
       </c>
       <c r="I9" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J9" s="60" t="n">
         <v>733.25</v>
       </c>
-      <c r="J9" s="60" t="n">
-        <v>2199.75</v>
-      </c>
       <c r="K9" s="61" t="n">
-        <v>3</v>
+        <v>804</v>
       </c>
       <c r="L9" s="9" t="n">
         <v>804</v>
       </c>
-      <c r="M9" s="62" t="n">
+      <c r="M9" s="62" t="n"/>
+      <c r="N9" s="60" t="n">
         <v>2199.75</v>
       </c>
-      <c r="N9" s="60" t="n">
-        <v>2412</v>
-      </c>
-      <c r="O9" s="60" t="n"/>
+      <c r="O9" s="60" t="n">
+        <v>2199.75</v>
+      </c>
       <c r="P9" s="13" t="n"/>
       <c r="Q9" s="61" t="n"/>
       <c r="R9" s="63" t="n"/>

</xml_diff>